<commit_message>
GT Login TC's Updated
</commit_message>
<xml_diff>
--- a/WEB/GujaratTitans/TestData/EmailDataList.xlsx
+++ b/WEB/GujaratTitans/TestData/EmailDataList.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="13680"/>
+    <workbookView windowWidth="30240" windowHeight="13620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$R$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$11</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="102">
   <si>
     <t>id</t>
   </si>
@@ -80,6 +80,9 @@
     <t>referral_code</t>
   </si>
   <si>
+    <t>state</t>
+  </si>
+  <si>
     <t>city</t>
   </si>
   <si>
@@ -89,6 +92,12 @@
     <t>caption</t>
   </si>
   <si>
+    <t>date_of_birth</t>
+  </si>
+  <si>
+    <t>fav_player</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -101,7 +110,7 @@
     <t>test1</t>
   </si>
   <si>
-    <t>MALE</t>
+    <t>Male</t>
   </si>
   <si>
     <t>888</t>
@@ -113,12 +122,21 @@
     <t>GT-VN0Q3T</t>
   </si>
   <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
     <t>Mumbai</t>
   </si>
   <si>
+    <t>India</t>
+  </si>
+  <si>
     <t>Aava De GT!</t>
   </si>
   <si>
+    <t>Shubman Gill</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -131,7 +149,7 @@
     <t>test2</t>
   </si>
   <si>
-    <t>FEMALE</t>
+    <t>Female</t>
   </si>
   <si>
     <t>19</t>
@@ -140,12 +158,18 @@
     <t>987672</t>
   </si>
   <si>
-    <t>Abu Dhabi</t>
+    <t>Gujarat</t>
+  </si>
+  <si>
+    <t>Surat</t>
   </si>
   <si>
     <t xml:space="preserve">Let's go GT😍 Aava De </t>
   </si>
   <si>
+    <t>Jos Buttler</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
@@ -158,7 +182,7 @@
     <t>test3</t>
   </si>
   <si>
-    <t>OTHER</t>
+    <t>Other</t>
   </si>
   <si>
     <t>975</t>
@@ -167,12 +191,18 @@
     <t>234546</t>
   </si>
   <si>
-    <t>Colombo</t>
+    <t>Goa</t>
+  </si>
+  <si>
+    <t>Kalangat</t>
   </si>
   <si>
     <t>Gujarat Titans, a team so grand, With bat in hand, they rule the land 🔥</t>
   </si>
   <si>
+    <t>Mohammed Siraj</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
@@ -191,12 +221,12 @@
     <t>731478</t>
   </si>
   <si>
-    <t>Lahore</t>
-  </si>
-  <si>
     <t>Aa varse pan Gt karse</t>
   </si>
   <si>
+    <t>Ishant Sharma</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
@@ -212,9 +242,6 @@
     <t>0</t>
   </si>
   <si>
-    <t>London</t>
-  </si>
-  <si>
     <t>6</t>
   </si>
   <si>
@@ -245,9 +272,6 @@
     <t>Recover Your Account.</t>
   </si>
   <si>
-    <t>Brisbane</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -264,9 +288,6 @@
   </si>
   <si>
     <t>acay ogkb bytx ftgi</t>
-  </si>
-  <si>
-    <t>Capetown</t>
   </si>
   <si>
     <t>8</t>
@@ -1527,7 +1548,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -1545,14 +1566,16 @@
     <col min="13" max="13" width="10.15625" style="1" customWidth="1"/>
     <col min="14" max="14" width="12.1015625" style="1" customWidth="1"/>
     <col min="15" max="15" width="9.140625" style="1"/>
-    <col min="16" max="16" width="10.9375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="1"/>
-    <col min="18" max="18" width="12.03125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="50" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="17" width="10.9375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" style="1"/>
+    <col min="19" max="19" width="12.03125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="50" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="21.21875" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:19">
+    <row r="1" ht="24" customHeight="1" spans="1:22">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1610,22 +1633,31 @@
       <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" ht="17" spans="1:19">
+    <row r="2" ht="17" spans="1:22">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
@@ -1634,43 +1666,54 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="R2" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="S2" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="6">
+        <v>22081995</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="3" ht="17" spans="1:19">
+    <row r="3" ht="17" spans="1:22">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -1679,43 +1722,54 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="M3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="N3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6" t="s">
-        <v>37</v>
+      <c r="T3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="U3" s="6">
+        <v>11101998</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="4" ht="17" spans="1:19">
+    <row r="4" ht="17" spans="1:22">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -1724,43 +1778,54 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="R4" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>54</v>
+      </c>
       <c r="S4" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="U4" s="6">
+        <v>22081995</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="5" ht="17" spans="1:19">
+    <row r="5" ht="17" spans="1:22">
       <c r="A5" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -1769,43 +1834,54 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="R5" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="S5" s="6" t="s">
-        <v>54</v>
+        <v>32</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="U5" s="6">
+        <v>22081995</v>
+      </c>
+      <c r="V5" s="6" t="s">
+        <v>64</v>
       </c>
     </row>
-    <row r="6" ht="17" spans="1:19">
+    <row r="6" ht="17" spans="1:22">
       <c r="A6" s="3" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -1814,311 +1890,377 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="T6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="M6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="P6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6" t="s">
-        <v>28</v>
+      <c r="U6" s="6">
+        <v>21101998</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="7" ht="17" spans="1:19">
+    <row r="7" ht="17" spans="1:22">
       <c r="A7" s="3" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G7" s="3">
         <v>993</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="R7" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>54</v>
+      </c>
       <c r="S7" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="U7" s="6">
+        <v>21101998</v>
+      </c>
+      <c r="V7" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="8" ht="17" spans="1:19">
+    <row r="8" ht="17" spans="1:22">
       <c r="A8" s="3" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="G8" s="3">
         <v>993</v>
       </c>
       <c r="H8" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>68</v>
-      </c>
       <c r="J8" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="M8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="U8" s="6">
+        <v>22081995</v>
+      </c>
+      <c r="V8" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" ht="17" spans="1:22">
+      <c r="A9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="P8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q8" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" ht="17" spans="1:19">
-      <c r="A9" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="G9" s="3">
         <v>993</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="M9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="U9" s="6">
+        <v>22081995</v>
+      </c>
+      <c r="V9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="N9" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6" t="s">
-        <v>54</v>
-      </c>
     </row>
-    <row r="10" ht="17" spans="1:19">
+    <row r="10" ht="17" spans="1:22">
       <c r="A10" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G10" s="3">
         <v>993</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="R10" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>54</v>
+      </c>
       <c r="S10" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="T10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="U10" s="6">
+        <v>10041997</v>
+      </c>
+      <c r="V10" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="11" ht="17" spans="1:19">
+    <row r="11" ht="17" spans="1:22">
       <c r="A11" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G11" s="3">
         <v>993</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="J11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="N11" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K11" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="O11" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Q11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="R11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="U11" s="6">
+        <v>15111994</v>
+      </c>
+      <c r="V11" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>